<commit_message>
Update activity DB and show 4 activity cards per row
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XHtQHkTAPgECYWK2jojrDb
</commit_message>
<xml_diff>
--- a/data/mathsw_db.xlsx
+++ b/data/mathsw_db.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gen0010-my.sharepoint.com/personal/nunchikochi_munjeong_gen_hs_kr/Documents/3_외부업무/2026수학SW전시분과운영/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="11_58A7DF869D40E9E6C5759D95C7622FFED6FC75D4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59D18F38-C09B-4EEF-9869-8A9778617537}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="11_58A7DF869D40E9E6C5759D95C7622FFED6FC75D4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FEE9D106-9074-49AE-833C-252A43A7E77B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DB" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">DB!$A$1:$E$8</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -127,6 +130,7 @@
       <sz val="13"/>
       <color theme="0"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -134,12 +138,14 @@
       <sz val="13"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -303,6 +309,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -532,142 +542,135 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="26.4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
-        <f t="shared" ref="A2:A8" si="0">ROW()-ROW($A$1)</f>
         <v>1</v>
       </c>
       <c r="B2" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="26.4" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
-        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="B3" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
-        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="B4" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>11</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="13.2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
-        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="B5" s="3">
         <v>2</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" ht="13.2" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
-        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="B6" s="3">
         <v>3</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" ht="13.2" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="26.4" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
-        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="B7" s="3">
         <v>3</v>
       </c>
       <c r="C7" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A8" s="3">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3">
+        <v>3</v>
+      </c>
+      <c r="C8" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D8" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E8" s="9" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A8" s="3">
-        <f t="shared" si="0"/>
-        <v>7</v>
-      </c>
-      <c r="B8" s="3">
-        <v>2</v>
-      </c>
-      <c r="C8" s="12" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>21</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="12" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="E3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="E4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="E5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="E6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="E7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="E8" r:id="rId7" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="E6" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="E7" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="E2" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="E3" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="E4" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="E8" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="E5" r:id="rId7" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>